<commit_message>
Update history and excel data
</commit_message>
<xml_diff>
--- a/ICT_AX_공고_최근1주일.xlsx
+++ b/ICT_AX_공고_최근1주일.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G84"/>
+  <dimension ref="A1:G105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -533,11 +533,7 @@
           <t>상세 접속 필요</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>https://www.nipa.kr/home/2-2/16712</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -570,11 +566,7 @@
           <t>상세 접속 필요</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>https://www.nipa.kr/home/2-2/16682</t>
-        </is>
-      </c>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -607,11 +599,7 @@
           <t>상세 접속 필요</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>https://www.nipa.kr/home/2-2/16680</t>
-        </is>
-      </c>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -644,11 +632,7 @@
           <t>상세 접속 필요</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>https://www.nipa.kr/home/2-2/16676</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -681,11 +665,7 @@
           <t>상세 접속 필요</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>https://www.nipa.kr/home/2-2/16675</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -718,11 +698,7 @@
           <t>상세 접속 필요</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>https://www.nipa.kr/home/2-2/16671</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -755,11 +731,7 @@
           <t>상세 접속 필요</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>https://www.nipa.kr/home/2-2/16668</t>
-        </is>
-      </c>
+      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -769,34 +741,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AI, 데이터</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>[전남] 2026년 AIㆍ데이터 스타트업 성장 지원사업 공고</t>
+          <t>전체</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-04-08 ~ 2026-04-29</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
-        </is>
-      </c>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -806,7 +774,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -816,24 +784,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026년 소공인 인프라시설 고도화 지원사업 모집 공고</t>
+          <t>전체</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-04-15 ~ 2026-04-30</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
-        </is>
-      </c>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -843,7 +807,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -853,24 +817,20 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026년 중소기업 혁신 유공 포상 후보자 모집 공고</t>
+          <t>전체</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-04-15 ~ 2026-05-14</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
-        </is>
-      </c>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -880,7 +840,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -890,24 +850,20 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026년 1차 일반 물류바우처 사업 참여기업 모집 공고</t>
+          <t>국가유산청</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-04-17 ~ 2026-05-06</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
-        </is>
-      </c>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -917,34 +873,30 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026년 2차 수출지원기반활용사업 참여기업 모집 공고(중소벤처기업부 소관 수출바우처사업)</t>
+          <t>대통령경호처</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-04-17 ~ 2026-05-06</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
-        </is>
-      </c>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -954,7 +906,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -964,24 +916,20 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026년 글로벌스케일업캠퍼스 인천 유니브-엑스(Univ. X) 참여기업 모집 공고</t>
+          <t>산업통상부</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-04-09 ~ 2026-04-27</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
-        </is>
-      </c>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -991,7 +939,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1001,24 +949,20 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026년 중소기업기술혁신개발사업 유망기술개발(구조혁신R&amp;D) 하반기 시행계획 공고</t>
+          <t>통일부</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-04-23 ~ 2026-07-06</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
-        </is>
-      </c>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1028,7 +972,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1038,24 +982,20 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>[전남] 2026년 가정간편식 제품 개발 지원사업 지원기업 모집 공고</t>
+          <t>2026년 산학연 연계 중소벤처 RBD 지원사업(STEP 4)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-04-08 ~ 2026-04-27</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
-        </is>
-      </c>
+          <t>2026-04-14 ~ 2026-05-14</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1065,7 +1005,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1075,24 +1015,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026년 아산시 단체관광객 유치 인센티브 지원계획 공고</t>
+          <t>2026년도 한국철도기술연구원 기본사업 신규 위탁과제 수행기관 공모(재공고)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>예산 소진시까지</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
-        </is>
-      </c>
+          <t>2026-04-13 ~ 2026-04-20</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1102,7 +1038,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1112,24 +1048,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026년 전북 글로벌게임센터 고도화 게임 제작지원사업 공고</t>
+          <t>2026년도 한국철도기술연구원 기본사업 신규 공동과제 수행기관 공모(재공고)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-04-08 ~ 2026-04-28</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
-        </is>
-      </c>
+          <t>2026-04-13 ~ 2026-04-20</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1139,7 +1071,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1149,24 +1081,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026년 K-뷰티ㆍ헬스케어 현지진출 프로그램  참여기업 모집 공고</t>
+          <t>2026년 KISTEP 기본사업 위탁연구과제 공모(과학기술 논문성과 분석연구(2011-2025))</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-04-07 ~ 2026-04-27</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
-        </is>
-      </c>
+          <t>2026-04-09 ~ 2026-05-08</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1176,34 +1104,30 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026년 혁신 프리미어 1000 녹색산업 우수기업 모집 공고</t>
+          <t>2026년 AI 기반 대학 과학기술 혁신사업(중앙거점) 신규과제 공모</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-04-08 ~ 2026-05-04</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
-        </is>
-      </c>
+          <t>2026-04-28 ~ 2026-05-12</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1213,34 +1137,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>[강원] 춘천시 2026년 생계형 1인 자영업자 사회보험료 지원 공고</t>
+          <t>2026년 AI 기반 대학 과학기술 혁신사업(AI4ST) 신규과제 공모</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-04-07 ~ 2027-01-30</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
-        </is>
-      </c>
+          <t>2026-05-07 ~ 2026-05-22</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1250,7 +1170,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1260,24 +1180,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>[강원] 춘천시 2026년 사회보험료(10인 미만) 지원 공고</t>
+          <t>2026년도 Net-zero구현초격차태양전지개발 사업 신규과제 공모</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-04-01 ~ 2027-01-30</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
-        </is>
-      </c>
+          <t>2026-01-23 ~ 2026-02-23</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1287,34 +1203,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026년도 전통시장 및 상점가 활성화 유공 포상 계획 공고</t>
+          <t>해외우수과학자유치사업 (Brain Pool / Brain Pool+) 2026년도 신규과제 공고</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-04-15 ~ 2026-05-11</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
-        </is>
-      </c>
+          <t>2026-02-12 ~ 2026-04-16</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1324,7 +1236,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1334,24 +1246,20 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>[충남] 아산시 2026년 3차 소규모사업장 대기방지시설 사물인터넷(IoT) 설치 지원사업 시행 계획 공고</t>
+          <t>2026년도 한국철도기술연구원 기본사업 신규 위탁과제 수행기관 공모</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-04-07 ~ 2026-05-08</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
-        </is>
-      </c>
+          <t>2026-03-27 ~ 2026-04-10</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1361,7 +1269,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1371,24 +1279,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>[울산] 2026년 베트남 종합 무역사절단 참가기업 모집 공고</t>
+          <t>2026년도 한국철도기술연구원 기본사업 신규 공동과제 수행기관 공모</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-04-07 ~ 2026-04-23</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
-        </is>
-      </c>
+          <t>2026-03-27 ~ 2026-04-10</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1398,7 +1302,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1408,24 +1312,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026년 북미 진출 GATE 프로그램 참여기업 모집 공고</t>
+          <t>더보기</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-03-23 ~ 2026-05-11</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
-        </is>
-      </c>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1435,7 +1335,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1445,24 +1345,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>[경기] 포천시 2026년 지역소공인육성사업 소공인특화지원센터 지원사업 공고</t>
+          <t>전체</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>세부사업별 상이</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
-        </is>
-      </c>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1472,7 +1368,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1482,24 +1378,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>[울산] 2026년 소상공인 재기지원자금 긴급 융자 지원계획 공고</t>
+          <t>더보기</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>선착순 접수</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
-        </is>
-      </c>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1509,7 +1401,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>기업마당</t>
+          <t>NTIS</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1519,24 +1411,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>[울산] 2026년 2차 소상공인 경영안정자금 긴급 융자 지원계획 공고</t>
+          <t>전체</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>확인필요</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>선착순 접수</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
-        </is>
-      </c>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1551,12 +1439,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>AI, 데이터</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>[전북] 2026년 전북특별자치도소상공인희망센터 컨설팅 지원 참여업체 모집 공고</t>
+          <t>[전남] 2026년 AIㆍ데이터 스타트업 성장 지원사업 공고</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1566,12 +1454,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-04-10 ~ 2026-10-31</t>
+          <t>2026-04-08 ~ 2026-04-29</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1481,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>[강원] 춘천시 2026년 1차 지식재산 국내분쟁 비용지원 사업 모집 공고</t>
+          <t>2026년 소공인 인프라시설 고도화 지원사업 모집 공고</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1603,12 +1491,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-04-10 ~ 2026-05-11</t>
+          <t>2026-04-15 ~ 2026-04-30</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
         </is>
       </c>
     </row>
@@ -1625,12 +1513,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>수출</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026년 중동 상황 대응 긴급 수출물류비 사업 대상 모집 공고</t>
+          <t>2026년 중소기업 혁신 유공 포상 후보자 모집 공고</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1640,12 +1528,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>예산 소진시까지</t>
+          <t>2026-04-15 ~ 2026-05-14</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
         </is>
       </c>
     </row>
@@ -1667,7 +1555,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>[강원] 2026년 지역혁신클러스터육성(비R&amp;D) 기업지원 프로그램 모집 공고</t>
+          <t>2026년 1차 일반 물류바우처 사업 참여기업 모집 공고</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1677,12 +1565,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-04-10 ~ 2026-04-24</t>
+          <t>2026-04-17 ~ 2026-05-06</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
         </is>
       </c>
     </row>
@@ -1699,12 +1587,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>[경북] 영천시 2026년 중소기업 고부가가치 전환육성 지원사업 공고</t>
+          <t>2026년 2차 수출지원기반활용사업 참여기업 모집 공고(중소벤처기업부 소관 수출바우처사업)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1714,12 +1602,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-04-10 ~ 2026-05-11</t>
+          <t>2026-04-17 ~ 2026-05-06</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1629,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>[경북] 영천시 2026년 영천기업 연구시설장비 바우처 지원사업 수혜기업 모집 공고</t>
+          <t>2026년 글로벌스케일업캠퍼스 인천 유니브-엑스(Univ. X) 참여기업 모집 공고</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1751,12 +1639,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>예산 소진시까지</t>
+          <t>2026-04-09 ~ 2026-04-27</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
         </is>
       </c>
     </row>
@@ -1778,7 +1666,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026년 디지털커머스 전문기관(소담스퀘어강원) 소상공인 모집 공고</t>
+          <t>2026년 중소기업기술혁신개발사업 유망기술개발(구조혁신R&amp;D) 하반기 시행계획 공고</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1788,12 +1676,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-04-13 ~ 2026-11-30</t>
+          <t>2026-04-23 ~ 2026-07-06</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
         </is>
       </c>
     </row>
@@ -1810,12 +1698,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AI, 실증</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>[호남권] 2026년 AI융합 지능형 농업생태계 구축사업 AI솔루션 실증 지원사업 통합 모집 공고</t>
+          <t>[전남] 2026년 가정간편식 제품 개발 지원사업 지원기업 모집 공고</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1825,12 +1713,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-04-10 ~ 2026-04-23</t>
+          <t>2026-04-08 ~ 2026-04-27</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1740,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>[서울] 2026년 지역수요 맞춤형 R&amp;D기획 지원사업 공고</t>
+          <t>2026년 아산시 단체관광객 유치 인센티브 지원계획 공고</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1862,12 +1750,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-04-14 ~ 2026-04-30</t>
+          <t>예산 소진시까지</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
         </is>
       </c>
     </row>
@@ -1889,7 +1777,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>[경북] 2026년 경북세일페스타 온라인 기획전 참여업체 모집 공고</t>
+          <t>2026년 전북 글로벌게임센터 고도화 게임 제작지원사업 공고</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1899,12 +1787,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>모집 완료시</t>
+          <t>2026-04-08 ~ 2026-04-28</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
         </is>
       </c>
     </row>
@@ -1926,7 +1814,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>[강원] 원주시 2026년 1차 중소기업 지식재산 국내 분쟁 지원 사업 모집 공고</t>
+          <t>2026년 K-뷰티ㆍ헬스케어 현지진출 프로그램  참여기업 모집 공고</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1936,12 +1824,12 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-04-10 ~ 2026-05-11</t>
+          <t>2026-04-07 ~ 2026-04-27</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
         </is>
       </c>
     </row>
@@ -1963,7 +1851,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>[강원] 강릉시 2026년 1차 중소기업 지식재산 국내 분쟁 지원 사업 모집 공고</t>
+          <t>2026년 혁신 프리미어 1000 녹색산업 우수기업 모집 공고</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1973,12 +1861,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-04-10 ~ 2026-05-11</t>
+          <t>2026-04-08 ~ 2026-05-04</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
         </is>
       </c>
     </row>
@@ -2000,7 +1888,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2026년 2분기 자랑스러운 중소기업인 접수 공고</t>
+          <t>[강원] 춘천시 2026년 생계형 1인 자영업자 사회보험료 지원 공고</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2010,12 +1898,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-05-08</t>
+          <t>2026-04-07 ~ 2027-01-30</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
         </is>
       </c>
     </row>
@@ -2037,7 +1925,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>2026년 생활용 섬유제품 제조역량강화사업 지원대상기업 모집 통합 공고</t>
+          <t>[강원] 춘천시 2026년 사회보험료(10인 미만) 지원 공고</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2047,12 +1935,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-04-10 ~ 2026-04-27</t>
+          <t>2026-04-01 ~ 2027-01-30</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
         </is>
       </c>
     </row>
@@ -2074,7 +1962,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>[경북] 2026년 산학연 연계 중소벤처 R&amp;BD 지원사업(산학연 연계 핵심 R&amp;D STEP 4) 시행계획 공고</t>
+          <t>2026년도 전통시장 및 상점가 활성화 유공 포상 계획 공고</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2084,12 +1972,12 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-04-14 ~ 2026-05-14</t>
+          <t>2026-04-15 ~ 2026-05-11</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=1</t>
         </is>
       </c>
     </row>
@@ -2111,7 +1999,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>[울산] 2026년 U-RISE 스타트업 캠퍼스 창업팀 모집 공고</t>
+          <t>[충남] 아산시 2026년 3차 소규모사업장 대기방지시설 사물인터넷(IoT) 설치 지원사업 시행 계획 공고</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2121,12 +2009,12 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-04-10 ~ 2026-04-30</t>
+          <t>2026-04-07 ~ 2026-05-08</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
         </is>
       </c>
     </row>
@@ -2148,7 +2036,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>[경기] 2026년 1차 경기스타트업플랫폼 투자연계 지원 프로그램 온라인 밋업위크 참여기업 모집 공고</t>
+          <t>[울산] 2026년 베트남 종합 무역사절단 참가기업 모집 공고</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2158,12 +2046,12 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-04-13 ~ 2026-04-27</t>
+          <t>2026-04-07 ~ 2026-04-23</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
         </is>
       </c>
     </row>
@@ -2185,7 +2073,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>[경기] 성남시 2026년 독일 뒤셀도르프 의료기기전시회(MEDICA 2026) 참가기업 모집 공고</t>
+          <t>2026년 북미 진출 GATE 프로그램 참여기업 모집 공고</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2195,12 +2083,12 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-04-14 ~ 2026-04-28</t>
+          <t>2026-03-23 ~ 2026-05-11</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2110,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>[경북] 2026년 2차 지역혁신 프로젝트 혁신창업ㆍ데스벨리 지원 공고</t>
+          <t>[경기] 포천시 2026년 지역소공인육성사업 소공인특화지원센터 지원사업 공고</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2232,12 +2120,12 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-04-20 ~ 2026-04-24</t>
+          <t>세부사업별 상이</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
         </is>
       </c>
     </row>
@@ -2259,22 +2147,22 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>[경북] 2026년 2차 중소기업 공공조달시장 진출 지원사업 수혜기업 모집 공고</t>
+          <t>[울산] 2026년 소상공인 재기지원자금 긴급 융자 지원계획 공고</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2026-04-08 ~ 2026-04-21</t>
+          <t>선착순 접수</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
         </is>
       </c>
     </row>
@@ -2296,22 +2184,22 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>[경북] 소공인 스케일업 지원사업 참여기업 모집 공고</t>
+          <t>[울산] 2026년 2차 소상공인 경영안정자금 긴급 융자 지원계획 공고</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-04-24</t>
+          <t>선착순 접수</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
         </is>
       </c>
     </row>
@@ -2333,22 +2221,22 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>[경남] 2026년 2차 우주항공분야 타깃마케팅(영국 2026 판보로에어쇼) 참가기업 모집 공고</t>
+          <t>[전북] 2026년 전북특별자치도소상공인희망센터 컨설팅 지원 참여업체 모집 공고</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-04-20</t>
+          <t>2026-04-10 ~ 2026-10-31</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
         </is>
       </c>
     </row>
@@ -2370,22 +2258,22 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>[광주] 2026년 해외 세일즈출장 및 바이어초청 지원사업 참가업체 모집 공고</t>
+          <t>[강원] 춘천시 2026년 1차 지식재산 국내분쟁 비용지원 사업 모집 공고</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>예산 소진시까지</t>
+          <t>2026-04-10 ~ 2026-05-11</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
         </is>
       </c>
     </row>
@@ -2402,27 +2290,27 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>수출</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>[강원] 동해시 2026년 자유무역지역 역량강화 기업지원사업 참여기업 모집 공고</t>
+          <t>2026년 중동 상황 대응 긴급 수출물류비 사업 대상 모집 공고</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-04-24</t>
+          <t>예산 소진시까지</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
         </is>
       </c>
     </row>
@@ -2444,22 +2332,22 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2026년 플라스틱 순환경제 해외진출 지원사업 모집 공고</t>
+          <t>[강원] 2026년 지역혁신클러스터육성(비R&amp;D) 기업지원 프로그램 모집 공고</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-05-06</t>
+          <t>2026-04-10 ~ 2026-04-24</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
         </is>
       </c>
     </row>
@@ -2481,22 +2369,22 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>[광주] 2026년 융ㆍ복합 가전산업 기업 브랜드 강화 지원 사업 참여 기업 모집 공고(지역주도형 일자리 지원사업)</t>
+          <t>[경북] 영천시 2026년 중소기업 고부가가치 전환육성 지원사업 공고</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-04-23</t>
+          <t>2026-04-10 ~ 2026-05-11</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
         </is>
       </c>
     </row>
@@ -2518,22 +2406,22 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>[경기] 화성시 2026년 소상공인 클린케어 지원사업 시행 공고</t>
+          <t>[경북] 영천시 2026년 영천기업 연구시설장비 바우처 지원사업 수혜기업 모집 공고</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-05-01</t>
+          <t>예산 소진시까지</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
         </is>
       </c>
     </row>
@@ -2555,22 +2443,22 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>[경기] 2026년 경기가족친화 일하기 좋은 기업 인증 지원사업 공고</t>
+          <t>2026년 디지털커머스 전문기관(소담스퀘어강원) 소상공인 모집 공고</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-04-30</t>
+          <t>2026-04-13 ~ 2026-11-30</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
         </is>
       </c>
     </row>
@@ -2587,27 +2475,27 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>AI, 실증</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>[광주] 2026년 중소사업장 가족친화경영지원사업 모집 공고</t>
+          <t>[호남권] 2026년 AI융합 지능형 농업생태계 구축사업 AI솔루션 실증 지원사업 통합 모집 공고</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2026-04-10 ~ 2026-04-24</t>
+          <t>2026-04-10 ~ 2026-04-23</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
         </is>
       </c>
     </row>
@@ -2624,27 +2512,27 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>AI, 실증, 데이터</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>[경기] 2026년 산업데이터 표준 기반 AI솔루션 실증지원 수요기업 모집 공고(산업데이터 표준 확산 기반 구축 사업)</t>
+          <t>[서울] 2026년 지역수요 맞춤형 R&amp;D기획 지원사업 공고</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-05-08</t>
+          <t>2026-04-14 ~ 2026-04-30</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=2</t>
         </is>
       </c>
     </row>
@@ -2666,22 +2554,22 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>[대전] 2026년 해외통상사무소 주관 해외바이어 초청 비즈니스 상담회 공고</t>
+          <t>[경북] 2026년 경북세일페스타 온라인 기획전 참여업체 모집 공고</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>2026-04-03 ~ 2026-05-30</t>
+          <t>모집 완료시</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
         </is>
       </c>
     </row>
@@ -2703,22 +2591,22 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>[경북] 소공인 환경개선 지원사업 참여기업 모집 공고</t>
+          <t>[강원] 원주시 2026년 1차 중소기업 지식재산 국내 분쟁 지원 사업 모집 공고</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-04-24</t>
+          <t>2026-04-10 ~ 2026-05-11</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
         </is>
       </c>
     </row>
@@ -2740,22 +2628,22 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2026년 일본 도쿄 추계 IT 주간 전시회(Japan IT Week Autumn) 한국관 참가기업 모집 공고</t>
+          <t>[강원] 강릉시 2026년 1차 중소기업 지식재산 국내 분쟁 지원 사업 모집 공고</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-04-30</t>
+          <t>2026-04-10 ~ 2026-05-11</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
         </is>
       </c>
     </row>
@@ -2777,22 +2665,22 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>[경북] 소공인 온라인 콘텐츠 마케팅 지원사업 참여기업 모집 공고</t>
+          <t>2026년 2분기 자랑스러운 중소기업인 접수 공고</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-04-24</t>
+          <t>2026-04-06 ~ 2026-05-08</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
         </is>
       </c>
     </row>
@@ -2814,22 +2702,22 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>[대전] 2026년 디자인 라이선스 지원사업 모집 공고(대전인쇄소공인특화지원센터)</t>
+          <t>2026년 생활용 섬유제품 제조역량강화사업 지원대상기업 모집 통합 공고</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-04-17</t>
+          <t>2026-04-10 ~ 2026-04-27</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
         </is>
       </c>
     </row>
@@ -2851,22 +2739,22 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>2026년 홍콩 주얼리&amp;젬월드 전시회(Jewellery &amp; Gem WORLD Hong Kong) 한국관 참가기업 모집 공고</t>
+          <t>[경북] 2026년 산학연 연계 중소벤처 R&amp;BD 지원사업(산학연 연계 핵심 R&amp;D STEP 4) 시행계획 공고</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-04-24</t>
+          <t>2026-04-14 ~ 2026-05-14</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
         </is>
       </c>
     </row>
@@ -2888,22 +2776,22 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>[전북] 2026년 국내박람회 개별 참가 지원 참여기업 모집 공고</t>
+          <t>[울산] 2026년 U-RISE 스타트업 캠퍼스 창업팀 모집 공고</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-04-17</t>
+          <t>2026-04-10 ~ 2026-04-30</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
         </is>
       </c>
     </row>
@@ -2925,22 +2813,22 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>[대전] 2026년 ESG 경영환경 지원사업 참여기업 모집 공고(대전인쇄소공인특화지원센터)</t>
+          <t>[경기] 2026년 1차 경기스타트업플랫폼 투자연계 지원 프로그램 온라인 밋업위크 참여기업 모집 공고</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-04-17</t>
+          <t>2026-04-13 ~ 2026-04-27</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
         </is>
       </c>
     </row>
@@ -2962,22 +2850,22 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>[대전] 2026년 청년ㆍ인쇄 협업 프로젝트 참여기업 모집 공고(대전인쇄소공인특화지원센터)</t>
+          <t>[경기] 성남시 2026년 독일 뒤셀도르프 의료기기전시회(MEDICA 2026) 참가기업 모집 공고</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-04-17</t>
+          <t>2026-04-14 ~ 2026-04-28</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
         </is>
       </c>
     </row>
@@ -2999,22 +2887,22 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>[부산] 2026년 지산학 스케일업 지원사업 참여기업 모집 공고(지산학 연결중개 촉진 지원사업)</t>
+          <t>[경북] 2026년 2차 지역혁신 프로젝트 혁신창업ㆍ데스벨리 지원 공고</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2026-04-13 ~ 2026-04-20</t>
+          <t>2026-04-20 ~ 2026-04-24</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
         </is>
       </c>
     </row>
@@ -3036,7 +2924,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>[대전] 2026년 컨설팅 지원사업 참여기업 모집 공고(대전인쇄소공인특화지원센터)</t>
+          <t>[경북] 2026년 2차 중소기업 공공조달시장 진출 지원사업 수혜기업 모집 공고</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3046,12 +2934,12 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>예산 소진시까지</t>
+          <t>2026-04-08 ~ 2026-04-21</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
         </is>
       </c>
     </row>
@@ -3073,7 +2961,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>[전북] 2026년 기술닥터 프로그램 참여기업 지원 모집 공고</t>
+          <t>[경북] 소공인 스케일업 지원사업 참여기업 모집 공고</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3083,12 +2971,12 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>2026-05-04 ~ 2026-05-08</t>
+          <t>2026-04-06 ~ 2026-04-24</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
         </is>
       </c>
     </row>
@@ -3110,7 +2998,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>[부산] 2026년 1차 지산학 기술도입 지원사업 참여기업 모집 공고(지산학 연결중개 촉진 지원사업)</t>
+          <t>[경남] 2026년 2차 우주항공분야 타깃마케팅(영국 2026 판보로에어쇼) 참가기업 모집 공고</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3120,12 +3008,12 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>2026-04-13 ~ 2026-04-20</t>
+          <t>2026-04-06 ~ 2026-04-20</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
         </is>
       </c>
     </row>
@@ -3142,12 +3030,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ICT</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>[전북] ICT이노베이션스퀘어 확산사업 기업협력프로젝트 참여기업 모집 공고</t>
+          <t>[광주] 2026년 해외 세일즈출장 및 바이어초청 지원사업 참가업체 모집 공고</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3157,12 +3045,12 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-08-28</t>
+          <t>예산 소진시까지</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
         </is>
       </c>
     </row>
@@ -3184,7 +3072,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>2026년 글로벌기업산업기술연계R&amp;D 사업 신규지원 대상과제 공고</t>
+          <t>[강원] 동해시 2026년 자유무역지역 역량강화 기업지원사업 참여기업 모집 공고</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3194,12 +3082,12 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-06-12</t>
+          <t>2026-04-06 ~ 2026-04-24</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=3</t>
         </is>
       </c>
     </row>
@@ -3221,7 +3109,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>[충북] 2026년 천연물 사업 다각화 지원사업 참여기업 모집 공고</t>
+          <t>2026년 플라스틱 순환경제 해외진출 지원사업 모집 공고</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3231,12 +3119,12 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-04-30</t>
+          <t>2026-04-06 ~ 2026-05-06</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
         </is>
       </c>
     </row>
@@ -3258,7 +3146,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>2026년 통상변화대응지원사업 참여기업 모집 공고</t>
+          <t>[광주] 2026년 융ㆍ복합 가전산업 기업 브랜드 강화 지원 사업 참여 기업 모집 공고(지역주도형 일자리 지원사업)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3268,12 +3156,12 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>예산 소진시까지</t>
+          <t>2026-04-06 ~ 2026-04-23</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3183,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>[제주] 2026년 제주관광 콘텐츠 프로젝트 지원사업 모집 공고(지역산업맞춤형 일자리지원 사업)</t>
+          <t>[경기] 화성시 2026년 소상공인 클린케어 지원사업 시행 공고</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3305,12 +3193,12 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>2026-04-13 ~ 2026-04-24</t>
+          <t>2026-04-06 ~ 2026-05-01</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
         </is>
       </c>
     </row>
@@ -3332,7 +3220,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>[전북] 2026년 국내박람회 개별 참가 지원 참여기업 모집 공고(전북특별자치도 우수상품 판로 개척 지원)</t>
+          <t>[경기] 2026년 경기가족친화 일하기 좋은 기업 인증 지원사업 공고</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3342,12 +3230,12 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-04-17</t>
+          <t>2026-04-06 ~ 2026-04-30</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
         </is>
       </c>
     </row>
@@ -3369,7 +3257,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>[세종] 2026년 제품 공인인증ㆍ시험비 지원사업 참여 스타트업 모집 공고(개발완성수준(TRL) 승격 지원사업)</t>
+          <t>[광주] 2026년 중소사업장 가족친화경영지원사업 모집 공고</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -3379,12 +3267,12 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-04-17</t>
+          <t>2026-04-10 ~ 2026-04-24</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
         </is>
       </c>
     </row>
@@ -3401,12 +3289,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>AI, 실증, 데이터</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>[충북] 2026년 천연물 신제품 개발 및 시제품 제작 지원 참여기업 모집 공고</t>
+          <t>[경기] 2026년 산업데이터 표준 기반 AI솔루션 실증지원 수요기업 모집 공고(산업데이터 표준 확산 기반 구축 사업)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3416,12 +3304,12 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-04-30</t>
+          <t>2026-04-06 ~ 2026-05-08</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3331,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>2026년 초격차 스타트업 프로젝트 모두의 챌린지 팹리스 참여기업 모집 공고</t>
+          <t>[대전] 2026년 해외통상사무소 주관 해외바이어 초청 비즈니스 상담회 공고</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -3453,12 +3341,12 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>2026-04-14 ~ 2026-05-11</t>
+          <t>2026-04-03 ~ 2026-05-30</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
         </is>
       </c>
     </row>
@@ -3480,7 +3368,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>2026년 우주ㆍ항공ㆍ방산용 에너지 세라믹소재 개발 지원사업 기업모집 공고</t>
+          <t>[경북] 소공인 환경개선 지원사업 참여기업 모집 공고</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3490,12 +3378,12 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>2026-04-06 ~ 2026-04-19</t>
+          <t>2026-04-06 ~ 2026-04-24</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
         </is>
       </c>
     </row>
@@ -3517,20 +3405,797 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
+          <t>2026년 일본 도쿄 추계 IT 주간 전시회(Japan IT Week Autumn) 한국관 참가기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>2026-04-06 ~ 2026-04-30</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>[경북] 소공인 온라인 콘텐츠 마케팅 지원사업 참여기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>2026-04-06 ~ 2026-04-24</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>[대전] 2026년 디자인 라이선스 지원사업 모집 공고(대전인쇄소공인특화지원센터)</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>2026-04-06 ~ 2026-04-17</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>2026년 홍콩 주얼리&amp;젬월드 전시회(Jewellery &amp; Gem WORLD Hong Kong) 한국관 참가기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>2026-04-06 ~ 2026-04-24</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>[전북] 2026년 국내박람회 개별 참가 지원 참여기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>2026-04-06 ~ 2026-04-17</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>[대전] 2026년 ESG 경영환경 지원사업 참여기업 모집 공고(대전인쇄소공인특화지원센터)</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>2026-04-06 ~ 2026-04-17</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>[대전] 2026년 청년ㆍ인쇄 협업 프로젝트 참여기업 모집 공고(대전인쇄소공인특화지원센터)</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>2026-04-06 ~ 2026-04-17</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=4</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>[부산] 2026년 지산학 스케일업 지원사업 참여기업 모집 공고(지산학 연결중개 촉진 지원사업)</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>2026-04-13 ~ 2026-04-20</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>[대전] 2026년 컨설팅 지원사업 참여기업 모집 공고(대전인쇄소공인특화지원센터)</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>예산 소진시까지</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>[전북] 2026년 기술닥터 프로그램 참여기업 지원 모집 공고</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>2026-05-04 ~ 2026-05-08</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>[부산] 2026년 1차 지산학 기술도입 지원사업 참여기업 모집 공고(지산학 연결중개 촉진 지원사업)</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>2026-04-13 ~ 2026-04-20</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>ICT</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>[전북] ICT이노베이션스퀘어 확산사업 기업협력프로젝트 참여기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>2026-04-06 ~ 2026-08-28</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>2026년 글로벌기업산업기술연계R&amp;D 사업 신규지원 대상과제 공고</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>2026-04-06 ~ 2026-06-12</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>[충북] 2026년 천연물 사업 다각화 지원사업 참여기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>2026-04-06 ~ 2026-04-30</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>2026년 통상변화대응지원사업 참여기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>예산 소진시까지</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>[제주] 2026년 제주관광 콘텐츠 프로젝트 지원사업 모집 공고(지역산업맞춤형 일자리지원 사업)</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>2026-04-13 ~ 2026-04-24</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>[전북] 2026년 국내박람회 개별 참가 지원 참여기업 모집 공고(전북특별자치도 우수상품 판로 개척 지원)</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>2026-04-06 ~ 2026-04-17</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>[세종] 2026년 제품 공인인증ㆍ시험비 지원사업 참여 스타트업 모집 공고(개발완성수준(TRL) 승격 지원사업)</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>2026-04-06 ~ 2026-04-17</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>[충북] 2026년 천연물 신제품 개발 및 시제품 제작 지원 참여기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>2026-04-06 ~ 2026-04-30</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>2026년 초격차 스타트업 프로젝트 모두의 챌린지 팹리스 참여기업 모집 공고</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>2026-04-14 ~ 2026-05-11</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>2026년 우주ㆍ항공ㆍ방산용 에너지 세라믹소재 개발 지원사업 기업모집 공고</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>2026-04-06 ~ 2026-04-19</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>기업마당</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
           <t>2026년 1차 세라믹서포터즈사업화R&amp;D지원사업 수혜기업 모집 공고</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
+      <c r="E105" t="inlineStr">
         <is>
           <t>2026-04-14</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr">
+      <c r="F105" t="inlineStr">
         <is>
           <t>2026-04-06 ~ 2026-04-19</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr">
+      <c r="G105" t="inlineStr">
         <is>
           <t>https://www.bizinfo.go.kr/sii/siia/selectSIIA200View.do?rows=15&amp;cpage=5</t>
         </is>

</xml_diff>